<commit_message>
Update manuscript figures and supplementary materials
</commit_message>
<xml_diff>
--- a/manuscript_material/source_data/Source_Data_ED_Fig1.xlsx
+++ b/manuscript_material/source_data/Source_Data_ED_Fig1.xlsx
@@ -475,7 +475,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Agent traces (one event log per run)</t>
+          <t>Execution traces (one event log per run)</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -491,7 +491,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Galaxy runs with a detailed history snapshot</t>
+          <t>Galaxy-condition runs with a detailed analysis-history snapshot</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -529,7 +529,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>of which ended in an error state</t>
+          <t>of which Galaxy job errors</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -545,7 +545,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Calls to the Galaxy interface</t>
+          <t>Galaxy interface calls</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -577,7 +577,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Failures examined trace by trace</t>
+          <t>Runs adjudicated trace by trace</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -609,22 +609,22 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>configuration</t>
+          <t>model_configuration</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>environment</t>
+          <t>execution_condition</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>replicate</t>
+          <t>replicate_run</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>archived_score</t>
+          <t>reported_benchmark_score</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">

</xml_diff>